<commit_message>
fix: 2026년형 Streamlit API 경고 해결 및 최종 UI 최적화
</commit_message>
<xml_diff>
--- a/invoice_coupang_final.xlsx
+++ b/invoice_coupang_final.xlsx
@@ -125,7 +125,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1688,7 +1688,7 @@
       <c r="A40" s="1" t="n"/>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>환        율(적용 환율: 1,427.87)</t>
+          <t>환        율(하나은행 2026.03.31 최종 송금환율 기준)</t>
         </is>
       </c>
       <c r="C40" s="10" t="n"/>

</xml_diff>